<commit_message>
Add admin UI and rule tooling; extend API, engine, and tariff data
- Admin API, models, db migration, monitor, and rule parser
- Frontend admin pages and main index updates
- Refresh Trump tariffs workbook and validation report
- Expand requirements (httpx, beautifulsoup4, anthropic)

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/validation_report.xlsx
+++ b/validation_report.xlsx
@@ -1657,7 +1657,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.0% = $5.80 | Sec 232 Aluminum (FRNs): 50.0% = $0.00 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.36</t>
+          <t>Base MFN Rate: 2.0% = $5.80 | Sec 232 Aluminum (FRNs): 25.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.36</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Sec 232 Aluminum (FRNs): 50.0% applied to 0.0% aluminum content</t>
+          <t>Sec 232 Aluminum (FRNs): 25.0% applied to 0.0% aluminum content</t>
         </is>
       </c>
       <c r="S16" t="b">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.0% = $145.14 | Sec 232 Aluminum (FRNs): 50.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $9.07</t>
+          <t>Base MFN Rate: 2.0% = $145.14 | Sec 232 Aluminum (FRNs): 25.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $9.07</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Sec 232 Aluminum (FRNs): 50.0% applied to 0.0% aluminum content</t>
+          <t>Sec 232 Aluminum (FRNs): 25.0% applied to 0.0% aluminum content</t>
         </is>
       </c>
       <c r="S17" t="b">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.0% = $46.36 | Sec 232 Aluminum (FRNs): 50.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $2.90</t>
+          <t>Base MFN Rate: 2.0% = $46.36 | Sec 232 Aluminum (FRNs): 25.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $2.90</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Sec 232 Aluminum (FRNs): 50.0% applied to 0.0% aluminum content</t>
+          <t>Sec 232 Aluminum (FRNs): 25.0% applied to 0.0% aluminum content</t>
         </is>
       </c>
       <c r="S18" t="b">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.0% = $6.90 | Sec 232 Aluminum (FRNs): 50.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.43</t>
+          <t>Base MFN Rate: 2.0% = $6.90 | Sec 232 Aluminum (FRNs): 25.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.43</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Sec 232 Aluminum (FRNs): 50.0% applied to 0.0% aluminum content</t>
+          <t>Sec 232 Aluminum (FRNs): 25.0% applied to 0.0% aluminum content</t>
         </is>
       </c>
       <c r="S19" t="b">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 0.0% = $0.00 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.58</t>
+          <t>Base MFN Rate: 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.58</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr"/>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 5.8% = $4.06 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.09</t>
+          <t>Base MFN Rate: 5.8% = $4.06 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.09</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr"/>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.5% = $14.15 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.71</t>
+          <t>Base MFN Rate: 2.5% = $14.15 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.71</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr"/>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 0.0% = $0.00 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $46.70 | HMF: 0.125% = $16.85</t>
+          <t>Base MFN Rate: 0.0% = $0.00 | MPF: 0.3464% = $46.70 | HMF: 0.125% = $16.85</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr"/>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 5.0% = $29.45 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.74</t>
+          <t>Base MFN Rate: 5.0% = $29.45 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.74</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr"/>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.5% = $1042.00 | Sec 232 Aluminum (FRNs): 50.0% = $0.00 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $144.38 | HMF: 0.125% = $52.10</t>
+          <t>Base MFN Rate: 2.5% = $1042.00 | Sec 232 Aluminum (FRNs): 25.0% = $0.00 | MPF: 0.3464% = $144.38 | HMF: 0.125% = $52.10</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -2967,7 +2967,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Sec 232 Aluminum (FRNs): 50.0% applied to 0.0% aluminum content</t>
+          <t>Sec 232 Aluminum (FRNs): 25.0% applied to 0.0% aluminum content</t>
         </is>
       </c>
       <c r="S34" t="b">
@@ -3261,7 +3261,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.5% = $20.93 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $1.05</t>
+          <t>Base MFN Rate: 2.5% = $20.93 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $1.05</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr"/>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.5% = $139.78 | Sec 232 Aluminum (FRNs): 50.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $6.99</t>
+          <t>Base MFN Rate: 2.5% = $139.78 | Sec 232 Aluminum (FRNs): 25.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $6.99</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Sec 232 Aluminum (FRNs): 50.0% applied to 0.0% aluminum content</t>
+          <t>Sec 232 Aluminum (FRNs): 25.0% applied to 0.0% aluminum content</t>
         </is>
       </c>
       <c r="S40" t="b">
@@ -3549,7 +3549,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.5% = $115.70 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $5.79</t>
+          <t>Base MFN Rate: 2.5% = $115.70 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $5.79</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr"/>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.5% = $22.73 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $1.14</t>
+          <t>Base MFN Rate: 2.5% = $22.73 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $1.14</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr"/>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.5% = $1.12 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.06</t>
+          <t>Base MFN Rate: 2.5% = $1.12 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $0.06</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr"/>
@@ -3899,7 +3899,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 0.0% = $0.00 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $2.81</t>
+          <t>Base MFN Rate: 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $2.81</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr"/>
@@ -5659,7 +5659,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.5% = $59.98 | Sec 232 Aluminum (FRNs): 50.0% = $0.00 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $3.00</t>
+          <t>Base MFN Rate: 2.5% = $59.98 | Sec 232 Aluminum (FRNs): 25.0% = $0.00 | MPF: 0.3464% = $31.67 | HMF: 0.125% = $3.00</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
@@ -5669,7 +5669,7 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>Sec 232 Aluminum (FRNs): 50.0% applied to 0.0% aluminum content</t>
+          <t>Sec 232 Aluminum (FRNs): 25.0% applied to 0.0% aluminum content</t>
         </is>
       </c>
       <c r="S71" t="b">
@@ -5807,7 +5807,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>Base MFN Rate: 2.5% = $0.00 | Sec 232 Aluminum (FRNs): 50.0% = $0.00 | Sec 232 Auto Parts (FRNs): 0.0% = $0.00 | MPF: 0.3464% = $31.67</t>
+          <t>Base MFN Rate: 2.5% = $0.00 | Sec 232 Aluminum (FRNs): 25.0% = $0.00 | MPF: 0.3464% = $31.67</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
@@ -5817,7 +5817,7 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>Sec 232 Aluminum (FRNs): 50.0% applied to 0.0% aluminum content</t>
+          <t>Sec 232 Aluminum (FRNs): 25.0% applied to 0.0% aluminum content</t>
         </is>
       </c>
       <c r="S73" t="b">

</xml_diff>